<commit_message>
admin take installment & attendance issue fixed
</commit_message>
<xml_diff>
--- a/wwwroot/AttendanceFile/studentattendance.xlsx
+++ b/wwwroot/AttendanceFile/studentattendance.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>Report Month</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Wankar Computer Typing Insitute</t>
   </si>
   <si>
-    <t>ghan</t>
+    <t>Ghananad Shukla</t>
   </si>
   <si>
     <t>Present</t>
@@ -86,10 +86,7 @@
     <t>A</t>
   </si>
   <si>
-    <t>wankar</t>
-  </si>
-  <si>
-    <t>sankalp</t>
+    <t>Sankalp Shastri</t>
   </si>
   <si>
     <t>11:51 PM</t>
@@ -125,19 +122,61 @@
     <t>10:13 AM</t>
   </si>
   <si>
+    <t>1:04 PM</t>
+  </si>
+  <si>
+    <t>2:11 PM</t>
+  </si>
+  <si>
+    <t>3:19 PM</t>
+  </si>
+  <si>
+    <t>5:16 PM</t>
+  </si>
+  <si>
+    <t>10:57 PM</t>
+  </si>
+  <si>
+    <t>1:57 PM</t>
+  </si>
+  <si>
+    <t>4:50 PM</t>
+  </si>
+  <si>
+    <t>3:16 PM</t>
+  </si>
+  <si>
+    <t>1:43 PM</t>
+  </si>
+  <si>
     <t>6:10 PM</t>
   </si>
   <si>
     <t>3:48 PM</t>
   </si>
   <si>
-    <t>shri</t>
+    <t>5:56 PM</t>
+  </si>
+  <si>
+    <t>5:24 PM</t>
+  </si>
+  <si>
+    <t>Shrikant Wankar</t>
   </si>
   <si>
     <t>6:03 AM</t>
   </si>
   <si>
+    <t>4:42 PM</t>
+  </si>
+  <si>
     <t>7:06 AM</t>
+  </si>
+  <si>
+    <t>6:52 PM</t>
+  </si>
+  <si>
+    <t>Mohan Deshmukh</t>
   </si>
 </sst>
 </file>
@@ -1101,7 +1140,7 @@
         <v>5</v>
       </c>
       <c r="O10" s="14">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="P10" s="1" t="s">
         <v>6</v>
@@ -1128,7 +1167,7 @@
         <v>6</v>
       </c>
       <c r="X10" s="14">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
@@ -1341,31 +1380,71 @@
       <c r="A13" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
+      <c r="B13" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>28</v>
+      </c>
       <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
+      <c r="G13" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="J13" s="15" t="s">
+        <v>32</v>
+      </c>
       <c r="K13" s="15"/>
       <c r="L13" s="15"/>
-      <c r="M13" s="15"/>
-      <c r="N13" s="15"/>
-      <c r="O13" s="15"/>
+      <c r="M13" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="N13" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="O13" s="15" t="s">
+        <v>35</v>
+      </c>
       <c r="P13" s="15"/>
       <c r="Q13" s="15"/>
-      <c r="R13" s="15"/>
-      <c r="S13" s="15"/>
-      <c r="T13" s="15"/>
-      <c r="U13" s="15"/>
-      <c r="V13" s="15"/>
-      <c r="W13" s="15"/>
-      <c r="X13" s="15"/>
-      <c r="Y13" s="15"/>
-      <c r="Z13" s="15"/>
+      <c r="R13" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="S13" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="T13" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="U13" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="V13" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="W13" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="X13" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y13" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z13" s="15" t="s">
+        <v>44</v>
+      </c>
       <c r="AA13" s="15"/>
       <c r="AB13" s="15"/>
       <c r="AC13" s="15"/>
@@ -1379,9 +1458,13 @@
         <v>18</v>
       </c>
       <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
+      <c r="C14" s="15" t="s">
+        <v>45</v>
+      </c>
       <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
+      <c r="E14" s="15" t="s">
+        <v>28</v>
+      </c>
       <c r="F14" s="15"/>
       <c r="G14" s="15"/>
       <c r="H14" s="15"/>
@@ -1391,16 +1474,22 @@
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
       <c r="N14" s="15"/>
-      <c r="O14" s="15"/>
+      <c r="O14" s="15" t="s">
+        <v>46</v>
+      </c>
       <c r="P14" s="15"/>
       <c r="Q14" s="15"/>
       <c r="R14" s="15"/>
       <c r="S14" s="15"/>
       <c r="T14" s="15"/>
-      <c r="U14" s="15"/>
+      <c r="U14" s="15" t="s">
+        <v>47</v>
+      </c>
       <c r="V14" s="15"/>
       <c r="W14" s="15"/>
-      <c r="X14" s="15"/>
+      <c r="X14" s="15" t="s">
+        <v>48</v>
+      </c>
       <c r="Y14" s="15"/>
       <c r="Z14" s="15"/>
       <c r="AA14" s="15"/>
@@ -1419,7 +1508,7 @@
         <v>0</v>
       </c>
       <c r="C15" s="15">
-        <v>0</v>
+        <v>1085</v>
       </c>
       <c r="D15" s="15">
         <v>0</v>
@@ -1455,7 +1544,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="15">
-        <v>0</v>
+        <v>335</v>
       </c>
       <c r="P15" s="15">
         <v>0</v>
@@ -1473,7 +1562,7 @@
         <v>0</v>
       </c>
       <c r="U15" s="15">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="V15" s="15">
         <v>0</v>
@@ -1482,7 +1571,7 @@
         <v>0</v>
       </c>
       <c r="X15" s="15">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="Y15" s="15">
         <v>0</v>
@@ -1512,32 +1601,32 @@
     </row>
     <row r="16">
       <c r="A16" s="1"/>
-      <c r="B16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>23</v>
+      <c r="B16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>22</v>
       </c>
       <c r="F16" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="G16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="I16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="J16" s="18" t="s">
-        <v>23</v>
+      <c r="G16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="H16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="I16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="J16" s="16" t="s">
+        <v>22</v>
       </c>
       <c r="K16" s="18" t="s">
         <v>23</v>
@@ -1545,14 +1634,14 @@
       <c r="L16" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="M16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="N16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="O16" s="18" t="s">
-        <v>23</v>
+      <c r="M16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="N16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="O16" s="16" t="s">
+        <v>22</v>
       </c>
       <c r="P16" s="18" t="s">
         <v>23</v>
@@ -1560,32 +1649,32 @@
       <c r="Q16" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="R16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="S16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="T16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="U16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="V16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="W16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="X16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="Z16" s="18" t="s">
-        <v>23</v>
+      <c r="R16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="S16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="T16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="U16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="V16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="W16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="X16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z16" s="16" t="s">
+        <v>22</v>
       </c>
       <c r="AA16" s="18" t="s">
         <v>23</v>
@@ -1644,22 +1733,22 @@
     <row r="18">
       <c r="A18" s="1"/>
       <c r="B18" s="10" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="H18" s="1" t="s">
         <v>5</v>
@@ -1683,7 +1772,7 @@
         <v>5</v>
       </c>
       <c r="O18" s="14">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="P18" s="1" t="s">
         <v>6</v>
@@ -1710,7 +1799,7 @@
         <v>6</v>
       </c>
       <c r="X18" s="14">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="Y18" s="1"/>
       <c r="Z18" s="1"/>
@@ -1923,45 +2012,27 @@
       <c r="A21" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>28</v>
-      </c>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
       <c r="E21" s="15" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="F21" s="15"/>
-      <c r="G21" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="H21" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="I21" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="J21" s="15" t="s">
-        <v>33</v>
-      </c>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
       <c r="K21" s="15"/>
       <c r="L21" s="15"/>
-      <c r="M21" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="N21" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="O21" s="15" t="s">
-        <v>36</v>
-      </c>
+      <c r="M21" s="15"/>
+      <c r="N21" s="15"/>
+      <c r="O21" s="15"/>
       <c r="P21" s="15"/>
       <c r="Q21" s="15"/>
-      <c r="R21" s="15"/>
+      <c r="R21" s="15" t="s">
+        <v>51</v>
+      </c>
       <c r="S21" s="15"/>
       <c r="T21" s="15"/>
       <c r="U21" s="15"/>
@@ -1983,12 +2054,10 @@
         <v>18</v>
       </c>
       <c r="B22" s="15"/>
-      <c r="C22" s="15" t="s">
-        <v>37</v>
-      </c>
+      <c r="C22" s="15"/>
       <c r="D22" s="15"/>
       <c r="E22" s="15" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="F22" s="15"/>
       <c r="G22" s="15"/>
@@ -1999,12 +2068,12 @@
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
       <c r="N22" s="15"/>
-      <c r="O22" s="15" t="s">
-        <v>38</v>
-      </c>
+      <c r="O22" s="15"/>
       <c r="P22" s="15"/>
       <c r="Q22" s="15"/>
-      <c r="R22" s="15"/>
+      <c r="R22" s="15" t="s">
+        <v>53</v>
+      </c>
       <c r="S22" s="15"/>
       <c r="T22" s="15"/>
       <c r="U22" s="15"/>
@@ -2029,13 +2098,13 @@
         <v>0</v>
       </c>
       <c r="C23" s="15">
-        <v>1085</v>
+        <v>0</v>
       </c>
       <c r="D23" s="15">
         <v>0</v>
       </c>
       <c r="E23" s="15">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="F23" s="15">
         <v>0</v>
@@ -2065,7 +2134,7 @@
         <v>0</v>
       </c>
       <c r="O23" s="15">
-        <v>335</v>
+        <v>0</v>
       </c>
       <c r="P23" s="15">
         <v>0</v>
@@ -2074,7 +2143,7 @@
         <v>0</v>
       </c>
       <c r="R23" s="15">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="S23" s="15">
         <v>0</v>
@@ -2122,14 +2191,14 @@
     </row>
     <row r="24">
       <c r="A24" s="1"/>
-      <c r="B24" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="D24" s="16" t="s">
-        <v>22</v>
+      <c r="B24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="E24" s="16" t="s">
         <v>22</v>
@@ -2137,41 +2206,41 @@
       <c r="F24" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="G24" s="16" t="s">
+      <c r="G24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="H24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="I24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="J24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="K24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="L24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="M24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="N24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="O24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="P24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="R24" s="16" t="s">
         <v>22</v>
-      </c>
-      <c r="H24" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="I24" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="J24" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="K24" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="L24" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="M24" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="N24" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="O24" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="P24" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q24" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="R24" s="18" t="s">
-        <v>23</v>
       </c>
       <c r="S24" s="18" t="s">
         <v>23</v>
@@ -2254,22 +2323,22 @@
     <row r="26">
       <c r="A26" s="1"/>
       <c r="B26" s="10" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>5</v>
@@ -2293,7 +2362,7 @@
         <v>5</v>
       </c>
       <c r="O26" s="14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P26" s="1" t="s">
         <v>6</v>
@@ -2320,7 +2389,7 @@
         <v>6</v>
       </c>
       <c r="X26" s="14">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Y26" s="1"/>
       <c r="Z26" s="1"/>
@@ -2536,9 +2605,7 @@
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
       <c r="D29" s="15"/>
-      <c r="E29" s="15" t="s">
-        <v>40</v>
-      </c>
+      <c r="E29" s="15"/>
       <c r="F29" s="15"/>
       <c r="G29" s="15"/>
       <c r="H29" s="15"/>
@@ -2575,9 +2642,7 @@
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
       <c r="D30" s="15"/>
-      <c r="E30" s="15" t="s">
-        <v>41</v>
-      </c>
+      <c r="E30" s="15"/>
       <c r="F30" s="15"/>
       <c r="G30" s="15"/>
       <c r="H30" s="15"/>
@@ -2621,7 +2686,7 @@
         <v>0</v>
       </c>
       <c r="E31" s="15">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="F31" s="15">
         <v>0</v>
@@ -2717,8 +2782,8 @@
       <c r="D32" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="E32" s="16" t="s">
-        <v>22</v>
+      <c r="E32" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="F32" s="18" t="s">
         <v>23</v>

</xml_diff>